<commit_message>
changing main and adding misclassification error.
</commit_message>
<xml_diff>
--- a/InputData.xlsx
+++ b/InputData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="5028" windowHeight="7032"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23016" windowHeight="6516"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -331,15 +331,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1">
-        <v>185</v>
+        <v>100</v>
       </c>
       <c r="B1">
-        <v>109</v>
+        <v>137</v>
       </c>
       <c r="C1">
         <v>100</v>
@@ -347,10 +347,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>140</v>
+        <v>252</v>
       </c>
       <c r="B2">
-        <v>166</v>
+        <v>30</v>
       </c>
       <c r="C2">
         <v>100</v>
@@ -358,10 +358,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>274</v>
+        <v>136</v>
       </c>
       <c r="B3">
-        <v>167</v>
+        <v>109</v>
       </c>
       <c r="C3">
         <v>100</v>
@@ -369,10 +369,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>100</v>
+        <v>231</v>
       </c>
       <c r="B4">
-        <v>27</v>
+        <v>98</v>
       </c>
       <c r="C4">
         <v>100</v>
@@ -380,10 +380,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>22</v>
+        <v>199</v>
       </c>
       <c r="B5">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -391,10 +391,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="B6">
-        <v>270</v>
+        <v>196</v>
       </c>
       <c r="C6">
         <v>100</v>
@@ -402,21 +402,21 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>200</v>
+        <v>295</v>
       </c>
       <c r="B7">
-        <v>121</v>
+        <v>207</v>
       </c>
       <c r="C7">
-        <v>100</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>100</v>
+        <v>171</v>
       </c>
       <c r="B8">
-        <v>118</v>
+        <v>253</v>
       </c>
       <c r="C8">
         <v>100</v>
@@ -424,10 +424,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>125</v>
+        <v>69</v>
       </c>
       <c r="B9">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C9">
         <v>100</v>
@@ -435,10 +435,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>48</v>
+        <v>234</v>
       </c>
       <c r="B10">
-        <v>250</v>
+        <v>207</v>
       </c>
       <c r="C10">
         <v>100</v>
@@ -446,10 +446,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>185</v>
+        <v>3</v>
       </c>
       <c r="B11">
-        <v>235</v>
+        <v>215</v>
       </c>
       <c r="C11">
         <v>100</v>
@@ -457,10 +457,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>69</v>
+        <v>27</v>
       </c>
       <c r="B12">
-        <v>72</v>
+        <v>127</v>
       </c>
       <c r="C12">
         <v>100</v>
@@ -468,10 +468,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="B13">
-        <v>174</v>
+        <v>291</v>
       </c>
       <c r="C13">
         <v>100</v>
@@ -479,10 +479,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>237</v>
+        <v>272</v>
       </c>
       <c r="B14">
-        <v>39</v>
+        <v>256</v>
       </c>
       <c r="C14">
         <v>100</v>
@@ -490,21 +490,21 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>8</v>
+        <v>274</v>
       </c>
       <c r="B15">
-        <v>151</v>
+        <v>185</v>
       </c>
       <c r="C15">
-        <v>100</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>35</v>
+        <v>237</v>
       </c>
       <c r="B16">
-        <v>156</v>
+        <v>226</v>
       </c>
       <c r="C16">
         <v>100</v>
@@ -512,21 +512,21 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>65</v>
+        <v>223</v>
       </c>
       <c r="B17">
-        <v>87</v>
+        <v>201</v>
       </c>
       <c r="C17">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>179</v>
+        <v>214</v>
       </c>
       <c r="B18">
-        <v>207</v>
+        <v>176</v>
       </c>
       <c r="C18">
         <v>100</v>
@@ -534,10 +534,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>87</v>
+        <v>121</v>
       </c>
       <c r="B19">
-        <v>285</v>
+        <v>99</v>
       </c>
       <c r="C19">
         <v>100</v>
@@ -545,10 +545,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>234</v>
+        <v>175</v>
       </c>
       <c r="B20">
-        <v>81</v>
+        <v>219</v>
       </c>
       <c r="C20">
         <v>100</v>
@@ -556,10 +556,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>89</v>
+        <v>205</v>
       </c>
       <c r="B21">
-        <v>192</v>
+        <v>254</v>
       </c>
       <c r="C21">
         <v>100</v>
@@ -567,10 +567,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>207</v>
+        <v>64</v>
       </c>
       <c r="B22">
-        <v>253</v>
+        <v>267</v>
       </c>
       <c r="C22">
         <v>100</v>
@@ -578,10 +578,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>83</v>
+        <v>251</v>
       </c>
       <c r="B23">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C23">
         <v>100</v>
@@ -589,10 +589,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>279</v>
+        <v>125</v>
       </c>
       <c r="B24">
-        <v>151</v>
+        <v>102</v>
       </c>
       <c r="C24">
         <v>100</v>
@@ -600,10 +600,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>103</v>
+        <v>176</v>
       </c>
       <c r="B25">
-        <v>27</v>
+        <v>256</v>
       </c>
       <c r="C25">
         <v>100</v>
@@ -611,10 +611,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>282</v>
+        <v>114</v>
       </c>
       <c r="B26">
-        <v>102</v>
+        <v>141</v>
       </c>
       <c r="C26">
         <v>100</v>
@@ -622,10 +622,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>145</v>
+        <v>234</v>
       </c>
       <c r="B27">
-        <v>42</v>
+        <v>94</v>
       </c>
       <c r="C27">
         <v>100</v>
@@ -633,10 +633,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>117</v>
+        <v>38</v>
       </c>
       <c r="B28">
-        <v>38</v>
+        <v>106</v>
       </c>
       <c r="C28">
         <v>100</v>
@@ -644,10 +644,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>231</v>
+        <v>282</v>
       </c>
       <c r="B29">
-        <v>146</v>
+        <v>39</v>
       </c>
       <c r="C29">
         <v>100</v>
@@ -655,21 +655,21 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>21</v>
+        <v>181</v>
       </c>
       <c r="B30">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="C30">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="B31">
-        <v>225</v>
+        <v>273</v>
       </c>
       <c r="C31">
         <v>100</v>
@@ -677,21 +677,21 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
-        <v>17</v>
+        <v>198</v>
       </c>
       <c r="B32">
-        <v>87</v>
+        <v>133</v>
       </c>
       <c r="C32">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
-        <v>2</v>
+        <v>198</v>
       </c>
       <c r="B33">
-        <v>92</v>
+        <v>286</v>
       </c>
       <c r="C33">
         <v>100</v>
@@ -699,10 +699,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
-        <v>37</v>
+        <v>115</v>
       </c>
       <c r="B34">
-        <v>13</v>
+        <v>159</v>
       </c>
       <c r="C34">
         <v>100</v>
@@ -710,10 +710,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
-        <v>115</v>
+        <v>173</v>
       </c>
       <c r="B35">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="C35">
         <v>100</v>
@@ -721,10 +721,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
-        <v>96</v>
+        <v>294</v>
       </c>
       <c r="B36">
-        <v>170</v>
+        <v>7</v>
       </c>
       <c r="C36">
         <v>100</v>
@@ -732,10 +732,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37">
-        <v>136</v>
+        <v>275</v>
       </c>
       <c r="B37">
-        <v>98</v>
+        <v>200</v>
       </c>
       <c r="C37">
         <v>100</v>
@@ -743,10 +743,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38">
-        <v>101</v>
+        <v>136</v>
       </c>
       <c r="B38">
-        <v>270</v>
+        <v>37</v>
       </c>
       <c r="C38">
         <v>100</v>
@@ -754,10 +754,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39">
-        <v>275</v>
+        <v>133</v>
       </c>
       <c r="B39">
-        <v>209</v>
+        <v>236</v>
       </c>
       <c r="C39">
         <v>100</v>
@@ -765,10 +765,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40">
-        <v>273</v>
+        <v>30</v>
       </c>
       <c r="B40">
-        <v>248</v>
+        <v>192</v>
       </c>
       <c r="C40">
         <v>100</v>
@@ -776,10 +776,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41">
-        <v>212</v>
+        <v>129</v>
       </c>
       <c r="B41">
-        <v>16</v>
+        <v>116</v>
       </c>
       <c r="C41">
         <v>100</v>
@@ -787,21 +787,21 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42">
-        <v>230</v>
+        <v>290</v>
       </c>
       <c r="B42">
-        <v>50</v>
+        <v>152</v>
       </c>
       <c r="C42">
-        <v>100</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43">
-        <v>6</v>
+        <v>220</v>
       </c>
       <c r="B43">
-        <v>179</v>
+        <v>296</v>
       </c>
       <c r="C43">
         <v>100</v>
@@ -809,10 +809,10 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="B44">
-        <v>145</v>
+        <v>96</v>
       </c>
       <c r="C44">
         <v>100</v>
@@ -820,10 +820,10 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45">
-        <v>7</v>
+        <v>258</v>
       </c>
       <c r="B45">
-        <v>199</v>
+        <v>231</v>
       </c>
       <c r="C45">
         <v>100</v>
@@ -831,10 +831,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46">
-        <v>291</v>
+        <v>41</v>
       </c>
       <c r="B46">
-        <v>229</v>
+        <v>198</v>
       </c>
       <c r="C46">
         <v>100</v>
@@ -842,10 +842,10 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47">
-        <v>165</v>
+        <v>294</v>
       </c>
       <c r="B47">
-        <v>180</v>
+        <v>206</v>
       </c>
       <c r="C47">
         <v>100</v>
@@ -853,10 +853,10 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48">
-        <v>8</v>
+        <v>203</v>
       </c>
       <c r="B48">
-        <v>103</v>
+        <v>46</v>
       </c>
       <c r="C48">
         <v>100</v>
@@ -864,21 +864,21 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49">
-        <v>54</v>
+        <v>151</v>
       </c>
       <c r="B49">
-        <v>73</v>
+        <v>124</v>
       </c>
       <c r="C49">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="B50">
-        <v>219</v>
+        <v>261</v>
       </c>
       <c r="C50">
         <v>100</v>
@@ -886,10 +886,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51">
-        <v>254</v>
+        <v>146</v>
       </c>
       <c r="B51">
-        <v>239</v>
+        <v>58</v>
       </c>
       <c r="C51">
         <v>100</v>
@@ -897,10 +897,10 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52">
-        <v>133</v>
+        <v>248</v>
       </c>
       <c r="B52">
-        <v>92</v>
+        <v>238</v>
       </c>
       <c r="C52">
         <v>100</v>
@@ -908,10 +908,10 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53">
-        <v>105</v>
+        <v>243</v>
       </c>
       <c r="B53">
-        <v>113</v>
+        <v>153</v>
       </c>
       <c r="C53">
         <v>100</v>
@@ -919,10 +919,10 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54">
-        <v>229</v>
+        <v>99</v>
       </c>
       <c r="B54">
-        <v>115</v>
+        <v>299</v>
       </c>
       <c r="C54">
         <v>100</v>
@@ -930,10 +930,10 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55">
-        <v>225</v>
+        <v>93</v>
       </c>
       <c r="B55">
-        <v>297</v>
+        <v>35</v>
       </c>
       <c r="C55">
         <v>100</v>
@@ -941,21 +941,21 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56">
-        <v>67</v>
+        <v>277</v>
       </c>
       <c r="B56">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="C56">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57">
-        <v>128</v>
+        <v>35</v>
       </c>
       <c r="B57">
-        <v>176</v>
+        <v>201</v>
       </c>
       <c r="C57">
         <v>100</v>
@@ -963,10 +963,10 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58">
-        <v>193</v>
+        <v>26</v>
       </c>
       <c r="B58">
-        <v>292</v>
+        <v>200</v>
       </c>
       <c r="C58">
         <v>100</v>
@@ -974,10 +974,10 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59">
-        <v>101</v>
+        <v>170</v>
       </c>
       <c r="B59">
-        <v>281</v>
+        <v>181</v>
       </c>
       <c r="C59">
         <v>100</v>
@@ -985,10 +985,10 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60">
-        <v>217</v>
+        <v>242</v>
       </c>
       <c r="B60">
-        <v>129</v>
+        <v>170</v>
       </c>
       <c r="C60">
         <v>100</v>
@@ -996,10 +996,10 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61">
-        <v>103</v>
+        <v>204</v>
       </c>
       <c r="B61">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="C61">
         <v>100</v>
@@ -1007,10 +1007,10 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62">
-        <v>164</v>
+        <v>259</v>
       </c>
       <c r="B62">
-        <v>82</v>
+        <v>154</v>
       </c>
       <c r="C62">
         <v>100</v>
@@ -1018,21 +1018,21 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63">
-        <v>42</v>
+        <v>187</v>
       </c>
       <c r="B63">
-        <v>119</v>
+        <v>172</v>
       </c>
       <c r="C63">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64">
-        <v>88</v>
+        <v>261</v>
       </c>
       <c r="B64">
-        <v>149</v>
+        <v>259</v>
       </c>
       <c r="C64">
         <v>100</v>
@@ -1040,10 +1040,10 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="B65">
-        <v>81</v>
+        <v>159</v>
       </c>
       <c r="C65">
         <v>100</v>
@@ -1051,10 +1051,10 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66">
-        <v>131</v>
+        <v>98</v>
       </c>
       <c r="B66">
-        <v>233</v>
+        <v>159</v>
       </c>
       <c r="C66">
         <v>100</v>
@@ -1062,10 +1062,10 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67">
-        <v>98</v>
+        <v>130</v>
       </c>
       <c r="B67">
-        <v>149</v>
+        <v>106</v>
       </c>
       <c r="C67">
         <v>100</v>
@@ -1073,10 +1073,10 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68">
-        <v>37</v>
+        <v>178</v>
       </c>
       <c r="B68">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="C68">
         <v>100</v>
@@ -1084,10 +1084,10 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69">
-        <v>185</v>
+        <v>276</v>
       </c>
       <c r="B69">
-        <v>142</v>
+        <v>246</v>
       </c>
       <c r="C69">
         <v>100</v>
@@ -1095,12 +1095,342 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70">
-        <v>297</v>
+        <v>77</v>
       </c>
       <c r="B70">
-        <v>97</v>
+        <v>202</v>
       </c>
       <c r="C70">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71">
+        <v>131</v>
+      </c>
+      <c r="B71">
+        <v>246</v>
+      </c>
+      <c r="C71">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A72">
+        <v>265</v>
+      </c>
+      <c r="B72">
+        <v>91</v>
+      </c>
+      <c r="C72">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73">
+        <v>251</v>
+      </c>
+      <c r="B73">
+        <v>203</v>
+      </c>
+      <c r="C73">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74">
+        <v>209</v>
+      </c>
+      <c r="B74">
+        <v>280</v>
+      </c>
+      <c r="C74">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A75">
+        <v>293</v>
+      </c>
+      <c r="B75">
+        <v>150</v>
+      </c>
+      <c r="C75">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A76">
+        <v>158</v>
+      </c>
+      <c r="B76">
+        <v>149</v>
+      </c>
+      <c r="C76">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77">
+        <v>225</v>
+      </c>
+      <c r="B77">
+        <v>12</v>
+      </c>
+      <c r="C77">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78">
+        <v>148</v>
+      </c>
+      <c r="B78">
+        <v>221</v>
+      </c>
+      <c r="C78">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79">
+        <v>25</v>
+      </c>
+      <c r="B79">
+        <v>25</v>
+      </c>
+      <c r="C79">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80">
+        <v>263</v>
+      </c>
+      <c r="B80">
+        <v>231</v>
+      </c>
+      <c r="C80">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81">
+        <v>104</v>
+      </c>
+      <c r="B81">
+        <v>107</v>
+      </c>
+      <c r="C81">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82">
+        <v>215</v>
+      </c>
+      <c r="B82">
+        <v>189</v>
+      </c>
+      <c r="C82">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83">
+        <v>33</v>
+      </c>
+      <c r="B83">
+        <v>89</v>
+      </c>
+      <c r="C83">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84">
+        <v>287</v>
+      </c>
+      <c r="B84">
+        <v>18</v>
+      </c>
+      <c r="C84">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85">
+        <v>122</v>
+      </c>
+      <c r="B85">
+        <v>130</v>
+      </c>
+      <c r="C85">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A86">
+        <v>12</v>
+      </c>
+      <c r="B86">
+        <v>0</v>
+      </c>
+      <c r="C86">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A87">
+        <v>296</v>
+      </c>
+      <c r="B87">
+        <v>195</v>
+      </c>
+      <c r="C87">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88">
+        <v>39</v>
+      </c>
+      <c r="B88">
+        <v>294</v>
+      </c>
+      <c r="C88">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A89">
+        <v>46</v>
+      </c>
+      <c r="B89">
+        <v>255</v>
+      </c>
+      <c r="C89">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90">
+        <v>145</v>
+      </c>
+      <c r="B90">
+        <v>177</v>
+      </c>
+      <c r="C90">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A91">
+        <v>115</v>
+      </c>
+      <c r="B91">
+        <v>264</v>
+      </c>
+      <c r="C91">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A92">
+        <v>205</v>
+      </c>
+      <c r="B92">
+        <v>37</v>
+      </c>
+      <c r="C92">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A93">
+        <v>35</v>
+      </c>
+      <c r="B93">
+        <v>274</v>
+      </c>
+      <c r="C93">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A94">
+        <v>262</v>
+      </c>
+      <c r="B94">
+        <v>135</v>
+      </c>
+      <c r="C94">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A95">
+        <v>295</v>
+      </c>
+      <c r="B95">
+        <v>227</v>
+      </c>
+      <c r="C95">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A96">
+        <v>1</v>
+      </c>
+      <c r="B96">
+        <v>271</v>
+      </c>
+      <c r="C96">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A97">
+        <v>9</v>
+      </c>
+      <c r="B97">
+        <v>275</v>
+      </c>
+      <c r="C97">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A98">
+        <v>117</v>
+      </c>
+      <c r="B98">
+        <v>43</v>
+      </c>
+      <c r="C98">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A99">
+        <v>212</v>
+      </c>
+      <c r="B99">
+        <v>32</v>
+      </c>
+      <c r="C99">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A100">
+        <v>143</v>
+      </c>
+      <c r="B100">
+        <v>100</v>
+      </c>
+      <c r="C100">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
adding compare plot to main and compare loop for four algorithm.
</commit_message>
<xml_diff>
--- a/InputData.xlsx
+++ b/InputData.xlsx
@@ -336,10 +336,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="B1">
-        <v>137</v>
+        <v>58</v>
       </c>
       <c r="C1">
         <v>100</v>
@@ -347,10 +347,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>252</v>
+        <v>192</v>
       </c>
       <c r="B2">
-        <v>30</v>
+        <v>247</v>
       </c>
       <c r="C2">
         <v>100</v>
@@ -358,10 +358,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>136</v>
+        <v>21</v>
       </c>
       <c r="B3">
-        <v>109</v>
+        <v>223</v>
       </c>
       <c r="C3">
         <v>100</v>
@@ -369,10 +369,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>231</v>
+        <v>291</v>
       </c>
       <c r="B4">
-        <v>98</v>
+        <v>191</v>
       </c>
       <c r="C4">
         <v>100</v>
@@ -380,10 +380,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
+        <v>285</v>
+      </c>
+      <c r="B5">
         <v>199</v>
-      </c>
-      <c r="B5">
-        <v>194</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -391,10 +391,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>194</v>
+        <v>161</v>
       </c>
       <c r="B6">
-        <v>196</v>
+        <v>91</v>
       </c>
       <c r="C6">
         <v>100</v>
@@ -402,21 +402,21 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>295</v>
+        <v>247</v>
       </c>
       <c r="B7">
-        <v>207</v>
+        <v>3</v>
       </c>
       <c r="C7">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>171</v>
+        <v>245</v>
       </c>
       <c r="B8">
-        <v>253</v>
+        <v>213</v>
       </c>
       <c r="C8">
         <v>100</v>
@@ -424,21 +424,21 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>69</v>
+        <v>286</v>
       </c>
       <c r="B9">
-        <v>262</v>
+        <v>174</v>
       </c>
       <c r="C9">
-        <v>100</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>234</v>
+        <v>12</v>
       </c>
       <c r="B10">
-        <v>207</v>
+        <v>255</v>
       </c>
       <c r="C10">
         <v>100</v>
@@ -446,10 +446,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B11">
-        <v>215</v>
+        <v>50</v>
       </c>
       <c r="C11">
         <v>100</v>
@@ -457,10 +457,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>27</v>
+        <v>102</v>
       </c>
       <c r="B12">
-        <v>127</v>
+        <v>219</v>
       </c>
       <c r="C12">
         <v>100</v>
@@ -468,10 +468,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>101</v>
+        <v>299</v>
       </c>
       <c r="B13">
-        <v>291</v>
+        <v>256</v>
       </c>
       <c r="C13">
         <v>100</v>
@@ -479,10 +479,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>272</v>
+        <v>285</v>
       </c>
       <c r="B14">
-        <v>256</v>
+        <v>62</v>
       </c>
       <c r="C14">
         <v>100</v>
@@ -490,21 +490,21 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>274</v>
+        <v>126</v>
       </c>
       <c r="B15">
-        <v>185</v>
+        <v>59</v>
       </c>
       <c r="C15">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>237</v>
+        <v>138</v>
       </c>
       <c r="B16">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="C16">
         <v>100</v>
@@ -512,10 +512,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="B17">
-        <v>201</v>
+        <v>211</v>
       </c>
       <c r="C17">
         <v>100</v>
@@ -523,10 +523,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>214</v>
+        <v>278</v>
       </c>
       <c r="B18">
-        <v>176</v>
+        <v>235</v>
       </c>
       <c r="C18">
         <v>100</v>
@@ -534,10 +534,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>121</v>
+        <v>49</v>
       </c>
       <c r="B19">
-        <v>99</v>
+        <v>170</v>
       </c>
       <c r="C19">
         <v>100</v>
@@ -545,10 +545,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B20">
-        <v>219</v>
+        <v>38</v>
       </c>
       <c r="C20">
         <v>100</v>
@@ -556,10 +556,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>205</v>
+        <v>17</v>
       </c>
       <c r="B21">
-        <v>254</v>
+        <v>17</v>
       </c>
       <c r="C21">
         <v>100</v>
@@ -567,10 +567,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="B22">
-        <v>267</v>
+        <v>126</v>
       </c>
       <c r="C22">
         <v>100</v>
@@ -578,10 +578,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>251</v>
+        <v>131</v>
       </c>
       <c r="B23">
-        <v>268</v>
+        <v>86</v>
       </c>
       <c r="C23">
         <v>100</v>
@@ -589,10 +589,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>125</v>
+        <v>176</v>
       </c>
       <c r="B24">
-        <v>102</v>
+        <v>53</v>
       </c>
       <c r="C24">
         <v>100</v>
@@ -600,10 +600,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>176</v>
+        <v>227</v>
       </c>
       <c r="B25">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="C25">
         <v>100</v>
@@ -611,10 +611,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="B26">
-        <v>141</v>
+        <v>9</v>
       </c>
       <c r="C26">
         <v>100</v>
@@ -622,10 +622,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>234</v>
+        <v>30</v>
       </c>
       <c r="B27">
-        <v>94</v>
+        <v>34</v>
       </c>
       <c r="C27">
         <v>100</v>
@@ -633,10 +633,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>38</v>
+        <v>255</v>
       </c>
       <c r="B28">
-        <v>106</v>
+        <v>256</v>
       </c>
       <c r="C28">
         <v>100</v>
@@ -644,10 +644,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>282</v>
+        <v>296</v>
       </c>
       <c r="B29">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C29">
         <v>100</v>
@@ -655,10 +655,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>181</v>
+        <v>274</v>
       </c>
       <c r="B30">
-        <v>140</v>
+        <v>292</v>
       </c>
       <c r="C30">
         <v>100</v>
@@ -666,10 +666,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B31">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="C31">
         <v>100</v>
@@ -677,10 +677,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
-        <v>198</v>
+        <v>108</v>
       </c>
       <c r="B32">
-        <v>133</v>
+        <v>79</v>
       </c>
       <c r="C32">
         <v>100</v>
@@ -688,10 +688,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
-        <v>198</v>
+        <v>289</v>
       </c>
       <c r="B33">
-        <v>286</v>
+        <v>19</v>
       </c>
       <c r="C33">
         <v>100</v>
@@ -699,10 +699,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
-        <v>115</v>
+        <v>182</v>
       </c>
       <c r="B34">
-        <v>159</v>
+        <v>43</v>
       </c>
       <c r="C34">
         <v>100</v>
@@ -710,10 +710,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
-        <v>173</v>
+        <v>45</v>
       </c>
       <c r="B35">
-        <v>36</v>
+        <v>172</v>
       </c>
       <c r="C35">
         <v>100</v>
@@ -721,10 +721,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
-        <v>294</v>
+        <v>186</v>
       </c>
       <c r="B36">
-        <v>7</v>
+        <v>299</v>
       </c>
       <c r="C36">
         <v>100</v>
@@ -732,10 +732,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37">
-        <v>275</v>
+        <v>28</v>
       </c>
       <c r="B37">
-        <v>200</v>
+        <v>52</v>
       </c>
       <c r="C37">
         <v>100</v>
@@ -743,10 +743,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38">
-        <v>136</v>
+        <v>170</v>
       </c>
       <c r="B38">
-        <v>37</v>
+        <v>189</v>
       </c>
       <c r="C38">
         <v>100</v>
@@ -754,10 +754,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39">
-        <v>133</v>
+        <v>177</v>
       </c>
       <c r="B39">
-        <v>236</v>
+        <v>166</v>
       </c>
       <c r="C39">
         <v>100</v>
@@ -765,10 +765,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40">
-        <v>30</v>
+        <v>252</v>
       </c>
       <c r="B40">
-        <v>192</v>
+        <v>24</v>
       </c>
       <c r="C40">
         <v>100</v>
@@ -776,10 +776,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B41">
-        <v>116</v>
+        <v>132</v>
       </c>
       <c r="C41">
         <v>100</v>
@@ -787,21 +787,21 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42">
-        <v>290</v>
+        <v>278</v>
       </c>
       <c r="B42">
-        <v>152</v>
+        <v>34</v>
       </c>
       <c r="C42">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43">
-        <v>220</v>
+        <v>30</v>
       </c>
       <c r="B43">
-        <v>296</v>
+        <v>232</v>
       </c>
       <c r="C43">
         <v>100</v>
@@ -809,10 +809,10 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44">
-        <v>33</v>
+        <v>193</v>
       </c>
       <c r="B44">
-        <v>96</v>
+        <v>20</v>
       </c>
       <c r="C44">
         <v>100</v>
@@ -820,10 +820,10 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45">
-        <v>258</v>
+        <v>18</v>
       </c>
       <c r="B45">
-        <v>231</v>
+        <v>203</v>
       </c>
       <c r="C45">
         <v>100</v>
@@ -831,10 +831,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46">
-        <v>41</v>
+        <v>220</v>
       </c>
       <c r="B46">
-        <v>198</v>
+        <v>35</v>
       </c>
       <c r="C46">
         <v>100</v>
@@ -842,10 +842,10 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47">
-        <v>294</v>
+        <v>276</v>
       </c>
       <c r="B47">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="C47">
         <v>100</v>
@@ -853,10 +853,10 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48">
-        <v>203</v>
+        <v>169</v>
       </c>
       <c r="B48">
-        <v>46</v>
+        <v>194</v>
       </c>
       <c r="C48">
         <v>100</v>
@@ -864,10 +864,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49">
-        <v>151</v>
+        <v>176</v>
       </c>
       <c r="B49">
-        <v>124</v>
+        <v>272</v>
       </c>
       <c r="C49">
         <v>100</v>
@@ -875,10 +875,10 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50">
-        <v>93</v>
+        <v>23</v>
       </c>
       <c r="B50">
-        <v>261</v>
+        <v>149</v>
       </c>
       <c r="C50">
         <v>100</v>
@@ -886,10 +886,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51">
-        <v>146</v>
+        <v>214</v>
       </c>
       <c r="B51">
-        <v>58</v>
+        <v>116</v>
       </c>
       <c r="C51">
         <v>100</v>
@@ -897,10 +897,10 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52">
-        <v>248</v>
+        <v>75</v>
       </c>
       <c r="B52">
-        <v>238</v>
+        <v>125</v>
       </c>
       <c r="C52">
         <v>100</v>
@@ -908,10 +908,10 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53">
-        <v>243</v>
+        <v>76</v>
       </c>
       <c r="B53">
-        <v>153</v>
+        <v>281</v>
       </c>
       <c r="C53">
         <v>100</v>
@@ -919,10 +919,10 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54">
-        <v>99</v>
+        <v>272</v>
       </c>
       <c r="B54">
-        <v>299</v>
+        <v>224</v>
       </c>
       <c r="C54">
         <v>100</v>
@@ -930,10 +930,10 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="B55">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="C55">
         <v>100</v>
@@ -941,10 +941,10 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56">
-        <v>277</v>
+        <v>105</v>
       </c>
       <c r="B56">
-        <v>80</v>
+        <v>195</v>
       </c>
       <c r="C56">
         <v>100</v>
@@ -952,10 +952,10 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="B57">
-        <v>201</v>
+        <v>155</v>
       </c>
       <c r="C57">
         <v>100</v>
@@ -963,10 +963,10 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58">
-        <v>26</v>
+        <v>64</v>
       </c>
       <c r="B58">
-        <v>200</v>
+        <v>251</v>
       </c>
       <c r="C58">
         <v>100</v>
@@ -974,10 +974,10 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59">
-        <v>170</v>
+        <v>265</v>
       </c>
       <c r="B59">
-        <v>181</v>
+        <v>233</v>
       </c>
       <c r="C59">
         <v>100</v>
@@ -985,10 +985,10 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60">
-        <v>242</v>
+        <v>148</v>
       </c>
       <c r="B60">
-        <v>170</v>
+        <v>43</v>
       </c>
       <c r="C60">
         <v>100</v>
@@ -996,10 +996,10 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61">
-        <v>204</v>
+        <v>45</v>
       </c>
       <c r="B61">
-        <v>68</v>
+        <v>202</v>
       </c>
       <c r="C61">
         <v>100</v>
@@ -1007,10 +1007,10 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62">
-        <v>259</v>
+        <v>113</v>
       </c>
       <c r="B62">
-        <v>154</v>
+        <v>209</v>
       </c>
       <c r="C62">
         <v>100</v>
@@ -1018,10 +1018,10 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63">
-        <v>187</v>
+        <v>159</v>
       </c>
       <c r="B63">
-        <v>172</v>
+        <v>102</v>
       </c>
       <c r="C63">
         <v>100</v>
@@ -1029,10 +1029,10 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64">
-        <v>261</v>
+        <v>136</v>
       </c>
       <c r="B64">
-        <v>259</v>
+        <v>233</v>
       </c>
       <c r="C64">
         <v>100</v>
@@ -1040,10 +1040,10 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65">
-        <v>9</v>
+        <v>93</v>
       </c>
       <c r="B65">
-        <v>159</v>
+        <v>127</v>
       </c>
       <c r="C65">
         <v>100</v>
@@ -1051,10 +1051,10 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66">
-        <v>98</v>
+        <v>169</v>
       </c>
       <c r="B66">
-        <v>159</v>
+        <v>43</v>
       </c>
       <c r="C66">
         <v>100</v>
@@ -1062,10 +1062,10 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67">
-        <v>130</v>
+        <v>285</v>
       </c>
       <c r="B67">
-        <v>106</v>
+        <v>294</v>
       </c>
       <c r="C67">
         <v>100</v>
@@ -1073,10 +1073,10 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68">
-        <v>178</v>
+        <v>84</v>
       </c>
       <c r="B68">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="C68">
         <v>100</v>
@@ -1084,10 +1084,10 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69">
-        <v>276</v>
+        <v>231</v>
       </c>
       <c r="B69">
-        <v>246</v>
+        <v>53</v>
       </c>
       <c r="C69">
         <v>100</v>
@@ -1095,10 +1095,10 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70">
-        <v>77</v>
+        <v>296</v>
       </c>
       <c r="B70">
-        <v>202</v>
+        <v>37</v>
       </c>
       <c r="C70">
         <v>100</v>
@@ -1106,10 +1106,10 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71">
-        <v>131</v>
+        <v>55</v>
       </c>
       <c r="B71">
-        <v>246</v>
+        <v>226</v>
       </c>
       <c r="C71">
         <v>100</v>
@@ -1117,10 +1117,10 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72">
-        <v>265</v>
+        <v>52</v>
       </c>
       <c r="B72">
-        <v>91</v>
+        <v>224</v>
       </c>
       <c r="C72">
         <v>100</v>
@@ -1128,10 +1128,10 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="B73">
-        <v>203</v>
+        <v>101</v>
       </c>
       <c r="C73">
         <v>100</v>
@@ -1139,10 +1139,10 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74">
-        <v>209</v>
+        <v>287</v>
       </c>
       <c r="B74">
-        <v>280</v>
+        <v>133</v>
       </c>
       <c r="C74">
         <v>100</v>
@@ -1150,10 +1150,10 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75">
-        <v>293</v>
+        <v>141</v>
       </c>
       <c r="B75">
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="C75">
         <v>100</v>
@@ -1161,10 +1161,10 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76">
-        <v>158</v>
+        <v>134</v>
       </c>
       <c r="B76">
-        <v>149</v>
+        <v>183</v>
       </c>
       <c r="C76">
         <v>100</v>
@@ -1172,10 +1172,10 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77">
-        <v>225</v>
+        <v>63</v>
       </c>
       <c r="B77">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C77">
         <v>100</v>
@@ -1183,10 +1183,10 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78">
-        <v>148</v>
+        <v>179</v>
       </c>
       <c r="B78">
-        <v>221</v>
+        <v>140</v>
       </c>
       <c r="C78">
         <v>100</v>
@@ -1194,10 +1194,10 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="B79">
-        <v>25</v>
+        <v>159</v>
       </c>
       <c r="C79">
         <v>100</v>
@@ -1205,10 +1205,10 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80">
-        <v>263</v>
+        <v>76</v>
       </c>
       <c r="B80">
-        <v>231</v>
+        <v>111</v>
       </c>
       <c r="C80">
         <v>100</v>
@@ -1216,10 +1216,10 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81">
-        <v>104</v>
+        <v>40</v>
       </c>
       <c r="B81">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="C81">
         <v>100</v>
@@ -1227,21 +1227,21 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82">
-        <v>215</v>
+        <v>268</v>
       </c>
       <c r="B82">
-        <v>189</v>
+        <v>220</v>
       </c>
       <c r="C82">
-        <v>100</v>
+        <v>40</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="B83">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="C83">
         <v>100</v>
@@ -1249,10 +1249,10 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84">
-        <v>287</v>
+        <v>248</v>
       </c>
       <c r="B84">
-        <v>18</v>
+        <v>269</v>
       </c>
       <c r="C84">
         <v>100</v>
@@ -1260,10 +1260,10 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85">
-        <v>122</v>
+        <v>194</v>
       </c>
       <c r="B85">
-        <v>130</v>
+        <v>75</v>
       </c>
       <c r="C85">
         <v>100</v>
@@ -1271,10 +1271,10 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="B86">
-        <v>0</v>
+        <v>248</v>
       </c>
       <c r="C86">
         <v>100</v>
@@ -1282,10 +1282,10 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87">
-        <v>296</v>
+        <v>187</v>
       </c>
       <c r="B87">
-        <v>195</v>
+        <v>218</v>
       </c>
       <c r="C87">
         <v>100</v>
@@ -1293,10 +1293,10 @@
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88">
-        <v>39</v>
+        <v>182</v>
       </c>
       <c r="B88">
-        <v>294</v>
+        <v>8</v>
       </c>
       <c r="C88">
         <v>100</v>
@@ -1304,10 +1304,10 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89">
-        <v>46</v>
+        <v>11</v>
       </c>
       <c r="B89">
-        <v>255</v>
+        <v>213</v>
       </c>
       <c r="C89">
         <v>100</v>
@@ -1315,10 +1315,10 @@
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90">
-        <v>145</v>
+        <v>39</v>
       </c>
       <c r="B90">
-        <v>177</v>
+        <v>127</v>
       </c>
       <c r="C90">
         <v>100</v>
@@ -1326,10 +1326,10 @@
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="B91">
-        <v>264</v>
+        <v>134</v>
       </c>
       <c r="C91">
         <v>100</v>
@@ -1337,10 +1337,10 @@
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92">
-        <v>205</v>
+        <v>0</v>
       </c>
       <c r="B92">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="C92">
         <v>100</v>
@@ -1348,10 +1348,10 @@
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="B93">
-        <v>274</v>
+        <v>202</v>
       </c>
       <c r="C93">
         <v>100</v>
@@ -1359,10 +1359,10 @@
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94">
-        <v>262</v>
+        <v>47</v>
       </c>
       <c r="B94">
-        <v>135</v>
+        <v>186</v>
       </c>
       <c r="C94">
         <v>100</v>
@@ -1370,10 +1370,10 @@
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95">
-        <v>295</v>
+        <v>55</v>
       </c>
       <c r="B95">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C95">
         <v>100</v>
@@ -1381,10 +1381,10 @@
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96">
-        <v>1</v>
+        <v>66</v>
       </c>
       <c r="B96">
-        <v>271</v>
+        <v>242</v>
       </c>
       <c r="C96">
         <v>100</v>
@@ -1392,10 +1392,10 @@
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97">
-        <v>9</v>
+        <v>96</v>
       </c>
       <c r="B97">
-        <v>275</v>
+        <v>89</v>
       </c>
       <c r="C97">
         <v>100</v>
@@ -1403,10 +1403,10 @@
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98">
-        <v>117</v>
+        <v>25</v>
       </c>
       <c r="B98">
-        <v>43</v>
+        <v>105</v>
       </c>
       <c r="C98">
         <v>100</v>
@@ -1414,10 +1414,10 @@
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99">
-        <v>212</v>
+        <v>234</v>
       </c>
       <c r="B99">
-        <v>32</v>
+        <v>99</v>
       </c>
       <c r="C99">
         <v>100</v>
@@ -1425,10 +1425,10 @@
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B100">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C100">
         <v>100</v>

</xml_diff>